<commit_message>
Fill new-SKU lead times from Group/Category logic (no more blanks)
The 39 new/renamed SKUs had blank Lead Time Override. Rather than let them
fall back to warehouse defaults, assign each the mode lead time of its
(Group, Category) cohort — the pattern the catalog already follows:

- Group 1 Miami-produced, EO/PA  -> 7   (23 SKUs: PD-LAVENDER/PEPPERMINT/
  EUCALYPTUS/TEATREE lines, MX-SLEEP/STRESS/MIND/BEARD, EO-ROSEHIP-5ml,
  PA-BUMP-1oz)
- Group 2 kits, GK                -> 10  (12 SKUs: GK0541/GK0715 components)
- Group 3 China direct, NC        -> 30  (4 SKUs: NC4390/4394/4395/4396)

Every catalog row now carries an explicit lead time; 0 blanks. Totals on
today's FBA unchanged at the account level (Miami 2,630 / China 6,610) since
most new SKUs aren't in FBA yet, but future restocks now use the right lead.
</commit_message>
<xml_diff>
--- a/automation/catalog.xlsx
+++ b/automation/catalog.xlsx
@@ -1491,6 +1491,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K20" t="n">
+        <v>7</v>
+      </c>
       <c r="L20" t="n">
         <v>45</v>
       </c>
@@ -2071,6 +2074,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K32" t="n">
+        <v>7</v>
+      </c>
       <c r="L32" t="n">
         <v>45</v>
       </c>
@@ -2950,6 +2956,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K50" t="n">
+        <v>7</v>
+      </c>
       <c r="L50" t="n">
         <v>45</v>
       </c>
@@ -2996,6 +3005,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K51" t="n">
+        <v>7</v>
+      </c>
       <c r="L51" t="n">
         <v>45</v>
       </c>
@@ -3042,6 +3054,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K52" t="n">
+        <v>7</v>
+      </c>
       <c r="L52" t="n">
         <v>45</v>
       </c>
@@ -3088,6 +3103,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K53" t="n">
+        <v>7</v>
+      </c>
       <c r="L53" t="n">
         <v>45</v>
       </c>
@@ -3134,6 +3152,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K54" t="n">
+        <v>7</v>
+      </c>
       <c r="L54" t="n">
         <v>45</v>
       </c>
@@ -3180,6 +3201,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K55" t="n">
+        <v>7</v>
+      </c>
       <c r="L55" t="n">
         <v>45</v>
       </c>
@@ -3226,6 +3250,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K56" t="n">
+        <v>7</v>
+      </c>
       <c r="L56" t="n">
         <v>45</v>
       </c>
@@ -3272,6 +3299,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K57" t="n">
+        <v>7</v>
+      </c>
       <c r="L57" t="n">
         <v>45</v>
       </c>
@@ -3318,6 +3348,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K58" t="n">
+        <v>7</v>
+      </c>
       <c r="L58" t="n">
         <v>45</v>
       </c>
@@ -3364,6 +3397,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K59" t="n">
+        <v>7</v>
+      </c>
       <c r="L59" t="n">
         <v>45</v>
       </c>
@@ -3410,6 +3446,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K60" t="n">
+        <v>7</v>
+      </c>
       <c r="L60" t="n">
         <v>45</v>
       </c>
@@ -3456,6 +3495,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K61" t="n">
+        <v>7</v>
+      </c>
       <c r="L61" t="n">
         <v>45</v>
       </c>
@@ -3502,6 +3544,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K62" t="n">
+        <v>7</v>
+      </c>
       <c r="L62" t="n">
         <v>45</v>
       </c>
@@ -3548,6 +3593,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K63" t="n">
+        <v>7</v>
+      </c>
       <c r="L63" t="n">
         <v>45</v>
       </c>
@@ -3594,6 +3642,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K64" t="n">
+        <v>7</v>
+      </c>
       <c r="L64" t="n">
         <v>45</v>
       </c>
@@ -3640,6 +3691,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K65" t="n">
+        <v>7</v>
+      </c>
       <c r="L65" t="n">
         <v>45</v>
       </c>
@@ -3681,6 +3735,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K66" t="n">
+        <v>7</v>
+      </c>
       <c r="L66" t="n">
         <v>45</v>
       </c>
@@ -3722,6 +3779,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K67" t="n">
+        <v>7</v>
+      </c>
       <c r="L67" t="n">
         <v>45</v>
       </c>
@@ -3763,6 +3823,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K68" t="n">
+        <v>7</v>
+      </c>
       <c r="L68" t="n">
         <v>45</v>
       </c>
@@ -3804,6 +3867,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K69" t="n">
+        <v>7</v>
+      </c>
       <c r="L69" t="n">
         <v>45</v>
       </c>
@@ -3992,6 +4058,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K73" t="n">
+        <v>7</v>
+      </c>
       <c r="L73" t="n">
         <v>45</v>
       </c>
@@ -4822,6 +4891,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K90" t="n">
+        <v>10</v>
+      </c>
       <c r="L90" t="n">
         <v>45</v>
       </c>
@@ -4873,6 +4945,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K91" t="n">
+        <v>10</v>
+      </c>
       <c r="L91" t="n">
         <v>45</v>
       </c>
@@ -4924,6 +4999,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K92" t="n">
+        <v>10</v>
+      </c>
       <c r="L92" t="n">
         <v>45</v>
       </c>
@@ -4975,6 +5053,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K93" t="n">
+        <v>10</v>
+      </c>
       <c r="L93" t="n">
         <v>45</v>
       </c>
@@ -5026,6 +5107,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K94" t="n">
+        <v>10</v>
+      </c>
       <c r="L94" t="n">
         <v>45</v>
       </c>
@@ -5077,6 +5161,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K95" t="n">
+        <v>10</v>
+      </c>
       <c r="L95" t="n">
         <v>45</v>
       </c>
@@ -5128,6 +5215,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K96" t="n">
+        <v>10</v>
+      </c>
       <c r="L96" t="n">
         <v>45</v>
       </c>
@@ -5179,6 +5269,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K97" t="n">
+        <v>10</v>
+      </c>
       <c r="L97" t="n">
         <v>45</v>
       </c>
@@ -5230,6 +5323,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K98" t="n">
+        <v>10</v>
+      </c>
       <c r="L98" t="n">
         <v>45</v>
       </c>
@@ -5281,6 +5377,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K99" t="n">
+        <v>10</v>
+      </c>
       <c r="L99" t="n">
         <v>45</v>
       </c>
@@ -5332,6 +5431,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K100" t="n">
+        <v>10</v>
+      </c>
       <c r="L100" t="n">
         <v>45</v>
       </c>
@@ -5383,6 +5485,9 @@
           <t>Miami</t>
         </is>
       </c>
+      <c r="K101" t="n">
+        <v>10</v>
+      </c>
       <c r="L101" t="n">
         <v>45</v>
       </c>
@@ -8409,6 +8514,9 @@
           <t>NC</t>
         </is>
       </c>
+      <c r="K157" t="n">
+        <v>30</v>
+      </c>
       <c r="L157" t="n">
         <v>45</v>
       </c>
@@ -8460,6 +8568,9 @@
           <t>NC</t>
         </is>
       </c>
+      <c r="K158" t="n">
+        <v>30</v>
+      </c>
       <c r="L158" t="n">
         <v>45</v>
       </c>
@@ -8511,6 +8622,9 @@
           <t>NC</t>
         </is>
       </c>
+      <c r="K159" t="n">
+        <v>30</v>
+      </c>
       <c r="L159" t="n">
         <v>45</v>
       </c>
@@ -8561,6 +8675,9 @@
         <is>
           <t>NC</t>
         </is>
+      </c>
+      <c r="K160" t="n">
+        <v>30</v>
       </c>
       <c r="L160" t="n">
         <v>45</v>

</xml_diff>